<commit_message>
feat: ajusta modelo de 3 abas, cálculo de marketplace e corrige testes de integração
</commit_message>
<xml_diff>
--- a/tests/fixtures/motor_precos_fixtures.xlsx
+++ b/tests/fixtures/motor_precos_fixtures.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="produtos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="concorrentes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meus Produtos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concorrentes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxas de Marketplace" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,71 +415,65 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>sku</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>nome</t>
+          <t>Meus Produtos</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>custo_base</t>
+          <t>Custo Base</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>preco_custo</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>margem_desejada</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>margem_minima</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>imposto_marketplace</t>
+          <t>Margem Mínima</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MOUSE-001</t>
+          <t>SKU001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Mouse Gamer</t>
+          <t>Produto Exemplo A</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>50</v>
       </c>
       <c r="D2" t="n">
-        <v>50</v>
-      </c>
-      <c r="E2" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SKU002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Produto Exemplo B</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>120</v>
+      </c>
+      <c r="D3" t="n">
         <v>0.2</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.1</v>
       </c>
     </row>
   </sheetData>
@@ -492,29 +487,126 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>sku</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>preco_concorrente</t>
+          <t>Concorrentes</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Preços Concorrentes</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Data da Coleta</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MOUSE-001</t>
+          <t>SKU001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Loja X</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SKU001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Loja Y</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>72</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Taxa Mínima</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Outros Custos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>80</v>
+        <v>0.14</v>
+      </c>
+      <c r="C2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Shopee</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>